<commit_message>
feat(randomization): enhance randomization scheme and slot management with new status choices and expandable UI elements
</commit_message>
<xml_diff>
--- a/src/staticfiles/study/templates/randomization_arms_template.xlsx
+++ b/src/staticfiles/study/templates/randomization_arms_template.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21735" windowHeight="12270"/>
+    <workbookView windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="randomization.arms" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Scheme Code</t>
   </si>
@@ -43,6 +43,12 @@
   <si>
     <t>Display Order</t>
   </si>
+  <si>
+    <t>Is Active</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
 </sst>
 </file>
 
@@ -54,14 +60,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_-* #,##0\ &quot;₫&quot;_-;\-* #,##0\ &quot;₫&quot;_-;_-* &quot;-&quot;\ &quot;₫&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -532,153 +531,154 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -999,15 +999,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="4" max="4" width="13.7142857142857" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="20.7142857142857" customWidth="1"/>
+    <col min="4" max="4" width="21.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="24.8571428571429" customWidth="1"/>
+    <col min="6" max="6" width="21" customWidth="1"/>
+    <col min="7" max="7" width="21.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1023,6 +1027,12 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>